<commit_message>
dataset con aglomerativo, kmeans ydbscan sin varias iteraciones
</commit_message>
<xml_diff>
--- a/Excel de proyecto.xlsx
+++ b/Excel de proyecto.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yarel\Documents\UAEH Nuevo nun\MINERIA DE DATOS\Proyecto Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{323370B3-0C46-48B4-A0BB-8B5A1885216D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D14BDE-03CC-4CAA-B71A-2B95E5B39422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{4D76F3F1-FCE3-4E5A-9C85-8B3952C92D55}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="1" xr2:uid="{4D76F3F1-FCE3-4E5A-9C85-8B3952C92D55}"/>
   </bookViews>
   <sheets>
     <sheet name="Estadisticas descriptivas DataS" sheetId="1" r:id="rId1"/>
+    <sheet name="Datos escalados" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="64">
   <si>
     <t>count</t>
   </si>
@@ -289,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -298,6 +299,9 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2357,4 +2361,1722 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D2F7633-919F-43DC-ADD3-3C6051DE796C}">
+  <dimension ref="B1:J59"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="H1" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I1" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D2" s="4">
+        <v>4.1294790000000002E-16</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F2" s="3">
+        <v>-3.972899</v>
+      </c>
+      <c r="G2" s="3">
+        <v>-0.66165700000000005</v>
+      </c>
+      <c r="H2" s="3">
+        <v>-0.18862200000000001</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.75744699999999998</v>
+      </c>
+      <c r="J2" s="3">
+        <v>5.9608280000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D3" s="4">
+        <v>7.4560030000000005E-17</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F3" s="3">
+        <v>-1.1600779999999999</v>
+      </c>
+      <c r="G3" s="3">
+        <v>-0.63789799999999997</v>
+      </c>
+      <c r="H3" s="3">
+        <v>-0.29189999999999999</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.35976399999999997</v>
+      </c>
+      <c r="J3" s="3">
+        <v>16.827549999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D4" s="4">
+        <v>-1.21877E-17</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-0.15571399999999999</v>
+      </c>
+      <c r="G4" s="3">
+        <v>-2.1968999999999999E-2</v>
+      </c>
+      <c r="H4" s="3">
+        <v>-2.5539999999999998E-3</v>
+      </c>
+      <c r="I4" s="3">
+        <v>1.7179E-2</v>
+      </c>
+      <c r="J4" s="3">
+        <v>198.95445799999999</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D5" s="4">
+        <v>-8.0653879999999997E-19</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F5" s="3">
+        <v>-0.19048699999999999</v>
+      </c>
+      <c r="G5" s="3">
+        <v>6.7500000000000004E-4</v>
+      </c>
+      <c r="H5" s="3">
+        <v>6.7500000000000004E-4</v>
+      </c>
+      <c r="I5" s="3">
+        <v>6.7500000000000004E-4</v>
+      </c>
+      <c r="J5" s="3">
+        <v>199.000326</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1.953616E-17</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F6" s="3">
+        <v>-0.211094</v>
+      </c>
+      <c r="G6" s="3">
+        <v>-1.9429999999999999E-2</v>
+      </c>
+      <c r="H6" s="3">
+        <v>3.9800000000000002E-4</v>
+      </c>
+      <c r="I6" s="3">
+        <v>2.0049000000000001E-2</v>
+      </c>
+      <c r="J6" s="3">
+        <v>198.883779</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D7" s="4">
+        <v>8.4596960000000002E-17</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F7" s="3">
+        <v>-0.960449</v>
+      </c>
+      <c r="G7" s="3">
+        <v>-0.60746299999999998</v>
+      </c>
+      <c r="H7" s="3">
+        <v>-0.25447599999999998</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0.27500400000000003</v>
+      </c>
+      <c r="J7" s="3">
+        <v>25.866534000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D8" s="4">
+        <v>-1.147077E-17</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F8" s="3">
+        <v>-0.85436000000000001</v>
+      </c>
+      <c r="G8" s="3">
+        <v>-0.59496300000000002</v>
+      </c>
+      <c r="H8" s="3">
+        <v>-7.6169000000000001E-2</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0.183228</v>
+      </c>
+      <c r="J8" s="3">
+        <v>29.235709</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D9" s="4">
+        <v>-2.0073849999999999E-17</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F9" s="3">
+        <v>-0.54687200000000002</v>
+      </c>
+      <c r="G9" s="3">
+        <v>-0.42652600000000002</v>
+      </c>
+      <c r="H9" s="3">
+        <v>-0.42652600000000002</v>
+      </c>
+      <c r="I9" s="3">
+        <v>-6.5486000000000003E-2</v>
+      </c>
+      <c r="J9" s="3">
+        <v>14.857500999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1.6130780000000001E-18</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F10" s="3">
+        <v>-0.30426799999999998</v>
+      </c>
+      <c r="G10" s="3">
+        <v>-0.30426799999999998</v>
+      </c>
+      <c r="H10" s="3">
+        <v>-0.30426799999999998</v>
+      </c>
+      <c r="I10" s="3">
+        <v>-6.0829000000000001E-2</v>
+      </c>
+      <c r="J10" s="3">
+        <v>21.848690999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1.3764930000000001E-16</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-5.3863890000000003</v>
+      </c>
+      <c r="G11" s="3">
+        <v>-8.2705000000000001E-2</v>
+      </c>
+      <c r="H11" s="3">
+        <v>0.13719000000000001</v>
+      </c>
+      <c r="I11" s="3">
+        <v>0.36309999999999998</v>
+      </c>
+      <c r="J11" s="3">
+        <v>4.1370380000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1.3764930000000001E-16</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F12" s="3">
+        <v>-3.2600419999999999</v>
+      </c>
+      <c r="G12" s="3">
+        <v>-0.641015</v>
+      </c>
+      <c r="H12" s="3">
+        <v>-0.11720999999999999</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0.93040100000000003</v>
+      </c>
+      <c r="J12" s="3">
+        <v>1.4542060000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D13" s="4">
+        <v>-3.7280009999999997E-17</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F13" s="3">
+        <v>-0.23644499999999999</v>
+      </c>
+      <c r="G13" s="3">
+        <v>-0.23644499999999999</v>
+      </c>
+      <c r="H13" s="3">
+        <v>-0.23644499999999999</v>
+      </c>
+      <c r="I13" s="3">
+        <v>-0.23644499999999999</v>
+      </c>
+      <c r="J13" s="3">
+        <v>4.2293130000000003</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F14" s="3">
+        <v>-0.46535900000000002</v>
+      </c>
+      <c r="G14" s="3">
+        <v>-0.46535900000000002</v>
+      </c>
+      <c r="H14" s="3">
+        <v>-0.46535900000000002</v>
+      </c>
+      <c r="I14" s="3">
+        <v>-0.46535900000000002</v>
+      </c>
+      <c r="J14" s="3">
+        <v>2.1488800000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D15" s="4">
+        <v>-3.4412320000000002E-17</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F15" s="3">
+        <v>-0.432948</v>
+      </c>
+      <c r="G15" s="3">
+        <v>-0.432948</v>
+      </c>
+      <c r="H15" s="3">
+        <v>-0.432948</v>
+      </c>
+      <c r="I15" s="3">
+        <v>-0.432948</v>
+      </c>
+      <c r="J15" s="3">
+        <v>2.3097470000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D16" s="4">
+        <v>-1.147077E-17</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F16" s="3">
+        <v>-0.24948699999999999</v>
+      </c>
+      <c r="G16" s="3">
+        <v>-0.24948699999999999</v>
+      </c>
+      <c r="H16" s="3">
+        <v>-0.24948699999999999</v>
+      </c>
+      <c r="I16" s="3">
+        <v>-0.24948699999999999</v>
+      </c>
+      <c r="J16" s="3">
+        <v>4.0082240000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D17" s="4">
+        <v>6.8824640000000005E-17</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F17" s="3">
+        <v>-0.47691099999999997</v>
+      </c>
+      <c r="G17" s="3">
+        <v>-0.47691099999999997</v>
+      </c>
+      <c r="H17" s="3">
+        <v>-0.47691099999999997</v>
+      </c>
+      <c r="I17" s="3">
+        <v>-0.47691099999999997</v>
+      </c>
+      <c r="J17" s="3">
+        <v>2.0968260000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D18" s="4">
+        <v>4.5883089999999998E-17</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F18" s="3">
+        <v>-0.51956599999999997</v>
+      </c>
+      <c r="G18" s="3">
+        <v>-0.51956599999999997</v>
+      </c>
+      <c r="H18" s="3">
+        <v>-0.51956599999999997</v>
+      </c>
+      <c r="I18" s="3">
+        <v>-0.51956599999999997</v>
+      </c>
+      <c r="J18" s="3">
+        <v>1.924682</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D19" s="4">
+        <v>6.8824640000000005E-17</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F19" s="3">
+        <v>-0.38928499999999999</v>
+      </c>
+      <c r="G19" s="3">
+        <v>-0.38928499999999999</v>
+      </c>
+      <c r="H19" s="3">
+        <v>-0.38928499999999999</v>
+      </c>
+      <c r="I19" s="3">
+        <v>-0.31747900000000001</v>
+      </c>
+      <c r="J19" s="3">
+        <v>5.0392279999999996</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B20" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D20" s="4">
+        <v>5.4486169999999998E-17</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F20" s="3">
+        <v>-0.29911100000000002</v>
+      </c>
+      <c r="G20" s="3">
+        <v>-0.18376400000000001</v>
+      </c>
+      <c r="H20" s="3">
+        <v>-0.12803500000000001</v>
+      </c>
+      <c r="I20" s="3">
+        <v>-3.9905000000000003E-2</v>
+      </c>
+      <c r="J20" s="3">
+        <v>77.047822999999994</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D21" s="4">
+        <v>-4.5883089999999998E-17</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F21" s="3">
+        <v>-0.504799</v>
+      </c>
+      <c r="G21" s="3">
+        <v>-0.27484500000000001</v>
+      </c>
+      <c r="H21" s="3">
+        <v>-0.123824</v>
+      </c>
+      <c r="I21" s="3">
+        <v>7.1899000000000005E-2</v>
+      </c>
+      <c r="J21" s="3">
+        <v>68.487645000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D22" s="4">
+        <v>-1.147077E-17</v>
+      </c>
+      <c r="E22" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F22" s="3">
+        <v>-0.23475499999999999</v>
+      </c>
+      <c r="G22" s="3">
+        <v>-0.23475499999999999</v>
+      </c>
+      <c r="H22" s="3">
+        <v>-0.21061099999999999</v>
+      </c>
+      <c r="I22" s="3">
+        <v>-9.8514000000000004E-2</v>
+      </c>
+      <c r="J22" s="3">
+        <v>14.308586</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B23" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1.8353240000000001E-16</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F23" s="3">
+        <v>-3.5073479999999999</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0.42413099999999998</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0.42413099999999998</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0.42413099999999998</v>
+      </c>
+      <c r="J23" s="3">
+        <v>0.42413099999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1.6059079999999999E-16</v>
+      </c>
+      <c r="E24" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F24" s="3">
+        <v>-1.9191780000000001</v>
+      </c>
+      <c r="G24" s="3">
+        <v>-0.63978299999999999</v>
+      </c>
+      <c r="H24" s="3">
+        <v>-0.10888</v>
+      </c>
+      <c r="I24" s="3">
+        <v>0.53070200000000001</v>
+      </c>
+      <c r="J24" s="3">
+        <v>4.3228400000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B25" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D25" s="4">
+        <v>-5.7353870000000003E-17</v>
+      </c>
+      <c r="E25" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F25" s="3">
+        <v>-0.98303600000000002</v>
+      </c>
+      <c r="G25" s="3">
+        <v>-0.98215600000000003</v>
+      </c>
+      <c r="H25" s="3">
+        <v>-8.2211999999999993E-2</v>
+      </c>
+      <c r="I25" s="3">
+        <v>0.82609399999999999</v>
+      </c>
+      <c r="J25" s="3">
+        <v>2.1943030000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D26" s="4">
+        <v>-4.8750790000000003E-17</v>
+      </c>
+      <c r="E26" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F26" s="3">
+        <v>-0.92759499999999995</v>
+      </c>
+      <c r="G26" s="3">
+        <v>-0.343528</v>
+      </c>
+      <c r="H26" s="3">
+        <v>-0.21340600000000001</v>
+      </c>
+      <c r="I26" s="3">
+        <v>5.9478000000000003E-2</v>
+      </c>
+      <c r="J26" s="3">
+        <v>48.000103000000003</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B27" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D27" s="4">
+        <v>-3.4412320000000002E-17</v>
+      </c>
+      <c r="E27" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F27" s="3">
+        <v>-2.3790140000000002</v>
+      </c>
+      <c r="G27" s="3">
+        <v>-0.571573</v>
+      </c>
+      <c r="H27" s="3">
+        <v>-0.20163600000000001</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0.352294</v>
+      </c>
+      <c r="J27" s="3">
+        <v>30.673518999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B28" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D28" s="4">
+        <v>3.7280009999999997E-17</v>
+      </c>
+      <c r="E28" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F28" s="3">
+        <v>-0.20258699999999999</v>
+      </c>
+      <c r="G28" s="3">
+        <v>-0.170214</v>
+      </c>
+      <c r="H28" s="3">
+        <v>-0.141792</v>
+      </c>
+      <c r="I28" s="3">
+        <v>-7.0864999999999997E-2</v>
+      </c>
+      <c r="J28" s="3">
+        <v>42.521194000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B29" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D29" s="4">
+        <v>2.8676930000000001E-18</v>
+      </c>
+      <c r="E29" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F29" s="3">
+        <v>-0.25176599999999999</v>
+      </c>
+      <c r="G29" s="3">
+        <v>-0.22495399999999999</v>
+      </c>
+      <c r="H29" s="3">
+        <v>-0.18351799999999999</v>
+      </c>
+      <c r="I29" s="3">
+        <v>-5.6772999999999997E-2</v>
+      </c>
+      <c r="J29" s="3">
+        <v>20.302961</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B30" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D30" s="4">
+        <v>-1.8640010000000001E-17</v>
+      </c>
+      <c r="E30" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F30" s="3">
+        <v>-0.26441199999999998</v>
+      </c>
+      <c r="G30" s="3">
+        <v>-0.223886</v>
+      </c>
+      <c r="H30" s="3">
+        <v>-0.173545</v>
+      </c>
+      <c r="I30" s="3">
+        <v>-4.9633999999999998E-2</v>
+      </c>
+      <c r="J30" s="3">
+        <v>34.566823999999997</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B31" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D31" s="4">
+        <v>3.638386E-17</v>
+      </c>
+      <c r="E31" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F31" s="3">
+        <v>-0.44939099999999998</v>
+      </c>
+      <c r="G31" s="3">
+        <v>-0.44939099999999998</v>
+      </c>
+      <c r="H31" s="3">
+        <v>-0.44939099999999998</v>
+      </c>
+      <c r="I31" s="3">
+        <v>-0.44939099999999998</v>
+      </c>
+      <c r="J31" s="3">
+        <v>2.2252320000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D32" s="4">
+        <v>4.713771E-17</v>
+      </c>
+      <c r="E32" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F32" s="3">
+        <v>-0.47866399999999998</v>
+      </c>
+      <c r="G32" s="3">
+        <v>-0.47866399999999998</v>
+      </c>
+      <c r="H32" s="3">
+        <v>-0.47866399999999998</v>
+      </c>
+      <c r="I32" s="3">
+        <v>-0.47866399999999998</v>
+      </c>
+      <c r="J32" s="3">
+        <v>2.0891500000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B33" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D33" s="4">
+        <v>5.0184630000000001E-17</v>
+      </c>
+      <c r="E33" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F33" s="3">
+        <v>-0.48045399999999999</v>
+      </c>
+      <c r="G33" s="3">
+        <v>-0.48045399999999999</v>
+      </c>
+      <c r="H33" s="3">
+        <v>-0.48045399999999999</v>
+      </c>
+      <c r="I33" s="3">
+        <v>-0.48045399999999999</v>
+      </c>
+      <c r="J33" s="3">
+        <v>2.0813640000000002</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B34" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D34" s="4">
+        <v>2.9393860000000003E-17</v>
+      </c>
+      <c r="E34" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F34" s="3">
+        <v>-0.47376099999999999</v>
+      </c>
+      <c r="G34" s="3">
+        <v>-0.47376099999999999</v>
+      </c>
+      <c r="H34" s="3">
+        <v>-0.47376099999999999</v>
+      </c>
+      <c r="I34" s="3">
+        <v>-0.47376099999999999</v>
+      </c>
+      <c r="J34" s="3">
+        <v>2.1107689999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B35" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D35" s="4">
+        <v>-3.4770779999999997E-17</v>
+      </c>
+      <c r="E35" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F35" s="3">
+        <v>-0.409827</v>
+      </c>
+      <c r="G35" s="3">
+        <v>-0.409827</v>
+      </c>
+      <c r="H35" s="3">
+        <v>-0.409827</v>
+      </c>
+      <c r="I35" s="3">
+        <v>-0.409827</v>
+      </c>
+      <c r="J35" s="3">
+        <v>2.4400550000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B36" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D36" s="4">
+        <v>-4.3732319999999999E-17</v>
+      </c>
+      <c r="E36" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F36" s="3">
+        <v>-0.25682100000000002</v>
+      </c>
+      <c r="G36" s="3">
+        <v>-0.25682100000000002</v>
+      </c>
+      <c r="H36" s="3">
+        <v>-0.25682100000000002</v>
+      </c>
+      <c r="I36" s="3">
+        <v>-0.25682100000000002</v>
+      </c>
+      <c r="J36" s="3">
+        <v>3.8937689999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B37" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D37" s="4">
+        <v>-5.0184630000000003E-18</v>
+      </c>
+      <c r="E37" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F37" s="3">
+        <v>-0.27232200000000001</v>
+      </c>
+      <c r="G37" s="3">
+        <v>-0.27232200000000001</v>
+      </c>
+      <c r="H37" s="3">
+        <v>-0.27232200000000001</v>
+      </c>
+      <c r="I37" s="3">
+        <v>-0.27232200000000001</v>
+      </c>
+      <c r="J37" s="3">
+        <v>3.6721210000000002</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B38" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D38" s="4">
+        <v>-6.3806180000000005E-17</v>
+      </c>
+      <c r="E38" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F38" s="3">
+        <v>-0.38811800000000002</v>
+      </c>
+      <c r="G38" s="3">
+        <v>-0.38811800000000002</v>
+      </c>
+      <c r="H38" s="3">
+        <v>-0.38811800000000002</v>
+      </c>
+      <c r="I38" s="3">
+        <v>-0.38811800000000002</v>
+      </c>
+      <c r="J38" s="3">
+        <v>2.5765359999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B39" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D39" s="4">
+        <v>0</v>
+      </c>
+      <c r="E39" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F39" s="3">
+        <v>-0.70197399999999999</v>
+      </c>
+      <c r="G39" s="3">
+        <v>-0.60671399999999998</v>
+      </c>
+      <c r="H39" s="3">
+        <v>-0.57501199999999997</v>
+      </c>
+      <c r="I39" s="3">
+        <v>0.21431600000000001</v>
+      </c>
+      <c r="J39" s="3">
+        <v>2.8231030000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B40" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C40" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D40" s="4">
+        <v>-3.36954E-17</v>
+      </c>
+      <c r="E40" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F40" s="3">
+        <v>-0.64293500000000003</v>
+      </c>
+      <c r="G40" s="3">
+        <v>-0.52908900000000003</v>
+      </c>
+      <c r="H40" s="3">
+        <v>-0.49116300000000002</v>
+      </c>
+      <c r="I40" s="3">
+        <v>4.3583999999999998E-2</v>
+      </c>
+      <c r="J40" s="3">
+        <v>3.5715750000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B41" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D41" s="4">
+        <v>1.7206160000000001E-16</v>
+      </c>
+      <c r="E41" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F41" s="3">
+        <v>-0.76671100000000003</v>
+      </c>
+      <c r="G41" s="3">
+        <v>-0.66544400000000004</v>
+      </c>
+      <c r="H41" s="3">
+        <v>-0.62492400000000004</v>
+      </c>
+      <c r="I41" s="3">
+        <v>0.41786400000000001</v>
+      </c>
+      <c r="J41" s="3">
+        <v>2.4940600000000002</v>
+      </c>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B42" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D42" s="4">
+        <v>-1.4768620000000001E-16</v>
+      </c>
+      <c r="E42" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F42" s="3">
+        <v>-0.75806099999999998</v>
+      </c>
+      <c r="G42" s="3">
+        <v>-0.661269</v>
+      </c>
+      <c r="H42" s="3">
+        <v>-0.62255099999999997</v>
+      </c>
+      <c r="I42" s="3">
+        <v>0.51490400000000003</v>
+      </c>
+      <c r="J42" s="3">
+        <v>2.3807420000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B43" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D43" s="4">
+        <v>8.6030800000000006E-17</v>
+      </c>
+      <c r="E43" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F43" s="3">
+        <v>-0.80928699999999998</v>
+      </c>
+      <c r="G43" s="3">
+        <v>-0.71047700000000003</v>
+      </c>
+      <c r="H43" s="3">
+        <v>-0.66844899999999996</v>
+      </c>
+      <c r="I43" s="3">
+        <v>0.57388700000000004</v>
+      </c>
+      <c r="J43" s="3">
+        <v>2.3969909999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B44" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D44" s="4">
+        <v>1.8353240000000001E-16</v>
+      </c>
+      <c r="E44" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F44" s="3">
+        <v>-3.7997779999999999</v>
+      </c>
+      <c r="G44" s="3">
+        <v>-0.40454400000000001</v>
+      </c>
+      <c r="H44" s="3">
+        <v>8.6448999999999998E-2</v>
+      </c>
+      <c r="I44" s="3">
+        <v>0.55674800000000002</v>
+      </c>
+      <c r="J44" s="3">
+        <v>4.7704380000000004</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B45" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D45" s="4">
+        <v>0</v>
+      </c>
+      <c r="E45" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F45" s="3">
+        <v>-5.2931210000000002</v>
+      </c>
+      <c r="G45" s="3">
+        <v>-0.63501799999999997</v>
+      </c>
+      <c r="H45" s="3">
+        <v>-1.9859999999999999E-3</v>
+      </c>
+      <c r="I45" s="3">
+        <v>0.603769</v>
+      </c>
+      <c r="J45" s="3">
+        <v>6.2780889999999996</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B46" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D46" s="4">
+        <v>4.5883089999999998E-17</v>
+      </c>
+      <c r="E46" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F46" s="3">
+        <v>-2.2735729999999998</v>
+      </c>
+      <c r="G46" s="3">
+        <v>-0.64495499999999995</v>
+      </c>
+      <c r="H46" s="3">
+        <v>-3.4543999999999998E-2</v>
+      </c>
+      <c r="I46" s="3">
+        <v>0.61132799999999998</v>
+      </c>
+      <c r="J46" s="3">
+        <v>6.647926</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B47" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D47" s="4">
+        <v>8.6030800000000006E-17</v>
+      </c>
+      <c r="E47" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F47" s="3">
+        <v>-1.5342309999999999</v>
+      </c>
+      <c r="G47" s="3">
+        <v>-0.64619099999999996</v>
+      </c>
+      <c r="H47" s="3">
+        <v>-0.117726</v>
+      </c>
+      <c r="I47" s="3">
+        <v>0.47351100000000002</v>
+      </c>
+      <c r="J47" s="3">
+        <v>15.545321</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B48" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D48" s="4">
+        <v>2.0647389999999999E-16</v>
+      </c>
+      <c r="E48" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F48" s="3">
+        <v>-3.5864150000000001</v>
+      </c>
+      <c r="G48" s="3">
+        <v>-0.43190600000000001</v>
+      </c>
+      <c r="H48" s="3">
+        <v>0.14918799999999999</v>
+      </c>
+      <c r="I48" s="3">
+        <v>0.61959699999999995</v>
+      </c>
+      <c r="J48" s="3">
+        <v>1.6711</v>
+      </c>
+    </row>
+    <row r="49" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B49" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C49" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D49" s="4">
+        <v>8.6030800000000006E-17</v>
+      </c>
+      <c r="E49" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F49" s="3">
+        <v>-1.8439080000000001</v>
+      </c>
+      <c r="G49" s="3">
+        <v>-0.65799399999999997</v>
+      </c>
+      <c r="H49" s="3">
+        <v>-5.0805999999999997E-2</v>
+      </c>
+      <c r="I49" s="3">
+        <v>0.61914499999999995</v>
+      </c>
+      <c r="J49" s="3">
+        <v>4.5600300000000002</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D50" s="4">
+        <v>1.1470769999999999E-16</v>
+      </c>
+      <c r="E50" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F50" s="3">
+        <v>-3.3845610000000002</v>
+      </c>
+      <c r="G50" s="3">
+        <v>-0.455146</v>
+      </c>
+      <c r="H50" s="3">
+        <v>4.7161000000000002E-2</v>
+      </c>
+      <c r="I50" s="3">
+        <v>0.55100800000000005</v>
+      </c>
+      <c r="J50" s="3">
+        <v>6.181076</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B51" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C51" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D51" s="4">
+        <v>-1.147077E-17</v>
+      </c>
+      <c r="E51" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F51" s="3">
+        <v>-1.338384</v>
+      </c>
+      <c r="G51" s="3">
+        <v>-0.63725900000000002</v>
+      </c>
+      <c r="H51" s="3">
+        <v>6.3865000000000005E-2</v>
+      </c>
+      <c r="I51" s="3">
+        <v>6.3865000000000005E-2</v>
+      </c>
+      <c r="J51" s="3">
+        <v>12.684101999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B52" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D52" s="4">
+        <v>-1.77797E-16</v>
+      </c>
+      <c r="E52" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F52" s="3">
+        <v>-3.053998</v>
+      </c>
+      <c r="G52" s="3">
+        <v>-0.63251999999999997</v>
+      </c>
+      <c r="H52" s="3">
+        <v>0.17463899999999999</v>
+      </c>
+      <c r="I52" s="3">
+        <v>0.98179799999999995</v>
+      </c>
+      <c r="J52" s="3">
+        <v>0.98179799999999995</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B53" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C53" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D53" s="4">
+        <v>5.0184630000000001E-17</v>
+      </c>
+      <c r="E53" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F53" s="3">
+        <v>-5.7974629999999996</v>
+      </c>
+      <c r="G53" s="3">
+        <v>-0.53911900000000001</v>
+      </c>
+      <c r="H53" s="3">
+        <v>4.8469999999999999E-2</v>
+      </c>
+      <c r="I53" s="3">
+        <v>0.56856399999999996</v>
+      </c>
+      <c r="J53" s="3">
+        <v>2.0319120000000002</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B54" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C54" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D54" s="4">
+        <v>2.2941550000000001E-17</v>
+      </c>
+      <c r="E54" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F54" s="3">
+        <v>-1.6468469999999999</v>
+      </c>
+      <c r="G54" s="3">
+        <v>-0.61338300000000001</v>
+      </c>
+      <c r="H54" s="3">
+        <v>7.5593999999999995E-2</v>
+      </c>
+      <c r="I54" s="3">
+        <v>0.76456999999999997</v>
+      </c>
+      <c r="J54" s="3">
+        <v>1.7980339999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B55" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C55" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D55" s="4">
+        <v>1.1470769999999999E-16</v>
+      </c>
+      <c r="E55" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F55" s="3">
+        <v>-9.3581109999999992</v>
+      </c>
+      <c r="G55" s="3">
+        <v>-0.18348999999999999</v>
+      </c>
+      <c r="H55" s="3">
+        <v>7.8642000000000004E-2</v>
+      </c>
+      <c r="I55" s="3">
+        <v>0.60290600000000005</v>
+      </c>
+      <c r="J55" s="3">
+        <v>1.12717</v>
+      </c>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B56" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C56" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D56" s="4">
+        <v>-6.9541570000000005E-17</v>
+      </c>
+      <c r="E56" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F56" s="3">
+        <v>-0.870807</v>
+      </c>
+      <c r="G56" s="3">
+        <v>-0.870807</v>
+      </c>
+      <c r="H56" s="3">
+        <v>-0.40819100000000003</v>
+      </c>
+      <c r="I56" s="3">
+        <v>0.67124499999999998</v>
+      </c>
+      <c r="J56" s="3">
+        <v>2.2132969999999998</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B57" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C57" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D57" s="4">
+        <v>-1.147077E-17</v>
+      </c>
+      <c r="E57" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F57" s="3">
+        <v>-4.036308</v>
+      </c>
+      <c r="G57" s="3">
+        <v>-0.26907599999999998</v>
+      </c>
+      <c r="H57" s="3">
+        <v>-0.26907599999999998</v>
+      </c>
+      <c r="I57" s="3">
+        <v>0.29600900000000002</v>
+      </c>
+      <c r="J57" s="3">
+        <v>3.4981559999999998</v>
+      </c>
+    </row>
+    <row r="58" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B58" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D58" s="4">
+        <v>-5.5203099999999999E-17</v>
+      </c>
+      <c r="E58" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F58" s="3">
+        <v>-1.810719</v>
+      </c>
+      <c r="G58" s="3">
+        <v>-0.92789600000000005</v>
+      </c>
+      <c r="H58" s="3">
+        <v>0.83774899999999997</v>
+      </c>
+      <c r="I58" s="3">
+        <v>0.83774899999999997</v>
+      </c>
+      <c r="J58" s="3">
+        <v>0.83774899999999997</v>
+      </c>
+    </row>
+    <row r="59" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B59" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C59" s="3">
+        <v>39644</v>
+      </c>
+      <c r="D59" s="4">
+        <v>5.0184630000000001E-17</v>
+      </c>
+      <c r="E59" s="3">
+        <v>1.000013</v>
+      </c>
+      <c r="F59" s="3">
+        <v>-0.68965799999999999</v>
+      </c>
+      <c r="G59" s="3">
+        <v>-0.68965799999999999</v>
+      </c>
+      <c r="H59" s="3">
+        <v>-0.68965799999999999</v>
+      </c>
+      <c r="I59" s="3">
+        <v>0.41511199999999998</v>
+      </c>
+      <c r="J59" s="3">
+        <v>3.7294239999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>